<commit_message>
Harden department boundary standards and regenerate handbooks
</commit_message>
<xml_diff>
--- a/tools/data/qms-terminology-dictionary.xlsx
+++ b/tools/data/qms-terminology-dictionary.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata labels" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role code &amp; JD link" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance hats" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Department code &amp; handbook link" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vai tro &amp; Chuc danh'!$A$1:$E$37</definedName>
@@ -4805,7 +4806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4815,316 +4816,481 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Thuật ngữ tiếng Anh</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Bản dịch tiếng Việt</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Dịch (Yes/No)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Sales and Customer Service Department</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Phòng Kinh doanh và Dịch vụ khách hàng</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Dùng cho mandate cấp phòng ban; không dùng thay vai trò phê duyệt hoặc người giữ cam kết thương mại cá nhân.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Engineering Department</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Phòng Kỹ thuật</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Dùng cho thiết kế công nghệ, baseline và release cấp chức năng; không dùng thay ENGM, DFM, PE hoặc CAM trong ô quyết định.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Production Department</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Phòng Sản xuất</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Dùng cho execution cấp xưởng; khi đi tới stop / restart / resource commitment phải truy về role code tương ứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Production Planning and Control Function</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Phân hệ Điều độ và Kiểm soát sản xuất</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Dùng khi đang nói tới planning, dispatching và WIP control như một phân hệ ổn định thuộc D-PROD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Quality Department</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Phòng Chất lượng</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Production Department</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Phòng Sản xuất</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Engineering Department</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Phòng Kỹ thuật</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Purchasing Department</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Phòng Mua hàng</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Warehouse Department</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Phòng Kho</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="n"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Dùng cho mandate chất lượng cấp chức năng; các quyết định hold / release / disposition vẫn phải về role code.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Sales Department</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Phòng Kinh doanh</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="n"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Supply Chain Department</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Phòng Chuỗi cung ứng</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dùng cho mô hình nguồn cung tổng thể; mua hàng, kho, tool crib và logistics là các phân hệ ổn định bên trong.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Purchasing Function</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Phân hệ Mua hàng</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Dùng cho sourcing, PO và supplier follow-up; không dùng thay BUY hoặc SCM khi đi tới cam kết với nhà cung cấp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Warehouse Function</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Phân hệ Kho</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Dùng cho receiving, put-away, location control và inventory integrity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tool Crib Function</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Phân hệ Kho dao cụ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Dùng cho quản lý dụng cụ cắt, preset, issue/return và tool life evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Logistics and Shipping Function</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Phân hệ Logistics và Giao vận</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Dùng cho booking, shipment documents, carrier handoff và track-and-trace sau xuất hàng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Finance Department</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Phòng Tài chính</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>HR Department</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Dùng cho mandate tài chính và kiểm soát ghi nhận; không dùng thay FIN, APAR hoặc GLP trong quyết định cá nhân.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Human Resources Department</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>Phòng Nhân sự</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>HR giữ nguyên viết tắt</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Maintenance Department</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Phòng Bảo trì</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Dùng cho workforce planning, hồ sơ nhân sự và điều phối đào tạo; sign-off năng lực chuyên môn vẫn phải quay về role quyết định thuộc D-PROD / D-ENG / D-QUAL / D-SCM / D-FIN / D-IT / D-EHS tùy công việc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>EHS Department</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Phòng An toàn - Môi trường</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>EHS giữ nguyên viết tắt</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Phòng EHS</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>EHS giữ nguyên viết tắt; dùng cho mandate an toàn, môi trường và emergency preparedness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>IT Department</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Phòng CNTT</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>IT giữ nguyên viết tắt</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Planning Department</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Phòng Kế hoạch</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>All departments</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Tất cả các phòng ban</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>IT giữ nguyên viết tắt; dùng cho hạ tầng, endpoint, access, backup và support nền tảng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ERP Administration Function</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Phân hệ Quản trị ERP</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Dùng cho quyền hệ thống, workflow, cấu hình, change log và integrity giao dịch ERP; không dùng thay ESA trong phê duyệt cá nhân.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Department coverage gap</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Khoảng trống bao phủ phòng ban</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Dùng khi công việc có thật nhưng handbook hoặc department code chưa bao phủ rõ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Subfunction coverage gap</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Khoảng trống bao phủ phân hệ</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Dùng khi cần tách một phân hệ ổn định lặp lại nhưng hệ thống chưa khai báo D-code tương ứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>JD gap</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Khoảng trống chức danh gắn JD</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Dùng khi công việc đi tới quyết định cá nhân nhưng hệ thống chưa có JD tương ứng; không được che bằng tên phòng ban.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E14"/>
@@ -5588,7 +5754,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/07-JD-Finance/jd-ap-ar-and-payments-accountant.html</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -5624,7 +5789,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-buyer-purchasing.html</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -5660,7 +5824,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/03-JD-Engineering/jd-cam-nc-programmer.html</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -5736,7 +5899,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-cleaning-and-packaging-supervisor.html</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -5772,7 +5934,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-cleaning-packaging-technician.html</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -5808,7 +5969,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/06-JD-Sales/jd-customer-service.html</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -5844,7 +6004,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-deburr-team-lead.html</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -5880,7 +6039,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-deburr-technician.html</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -5916,7 +6074,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/03-JD-Engineering/jd-dfm-engineer.html</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -5992,7 +6149,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/03-JD-Engineering/jd-engineering-lead-manager.html</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -6068,7 +6224,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/06-JD-Sales/jd-estimator.html</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -6104,7 +6259,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/07-JD-Finance/jd-finance-manager.html</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -6140,7 +6294,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/07-JD-Finance/jd-general-ledger-and-payroll-accountant.html</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -6176,7 +6329,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/08-JD-HR/jd-hr-manager.html</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -6212,7 +6364,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-internal-auditor-outsource.html</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -6288,7 +6439,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-logistics-shipping-coordinator.html</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -6324,7 +6474,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-metrology-and-calibration-specialist.html</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -6360,7 +6509,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-maintenance-technician.html</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -6396,7 +6544,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-cnc-operator.html</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -6472,7 +6619,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/03-JD-Engineering/jd-process-engineer.html</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -6548,7 +6694,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-production-planner.html</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -6624,7 +6769,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-qc-inspector-cmm-programmer-operator.html</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -6660,7 +6804,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-qc-inspector-lead.html</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -6696,7 +6839,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-quality-engineer.html</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -6772,7 +6914,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-supply-chain-manager.html</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -6808,7 +6949,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-setup-technician.html</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -6844,7 +6984,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-shift-leader.html</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -6880,7 +7019,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-tool-crib-tool-storekeeper.html</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -6916,7 +7054,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-warehouse-clerk.html</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -6952,7 +7089,6 @@
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-cnc-workshop-manager.html</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7223,4 +7359,835 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Department code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Department title English</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Tên tiếng Việt chuẩn</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Loại</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Parent department</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handbook path</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Lead roles</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Mandate summary</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Boundary / use note</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Coverage gap / expansion trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>D-EHS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EHS Department</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Phong EHS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-ehs-handbook.html</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EHS</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Bảo vệ con người, môi trường làm việc và tài sản vận hành bằng một hệ thống an toàn thực chiến: nhận diện mối nguy, giữ kỷ luật permit / LOTO, điều tra học từ sự cố và duy trì readiness cho tình huống khẩn cấp trong nhà máy job-order CNC.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>EHS giữ nguyên viết tắt; dùng cho mandate an toàn, môi trường và emergency preparedness.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD EHS Manager; EHS Specialist đang giữ phương pháp và điều phối chính, còn quyết định plant-wide shutdown hoặc reopening vẫn do CEO / PD giữ. | Nếu nhà máy mở thêm hoạt động rủi ro cao hoặc tăng tải compliance / contractor, cần xem xét mở vai trò quản lý EHS riêng thay vì giữ một chuyên viên đơn tuyến.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>D-ENG</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Engineering Department</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Phong Ky thuat</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-engineering-handbook.html</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ENGM, DFM, PE, CAM</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Biến yêu cầu kỹ thuật của khách hàng thành baseline gia công đáng tin cậy: đúng process, đúng chương trình, đúng control requirement và đủ dữ liệu để production, quality và planning có thể thực thi mà không phải suy diễn.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Dùng cho thiết kế công nghệ, baseline và release cấp chức năng; không dùng thay ENGM, DFM, PE hoặc CAM trong ô quyết định.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Hiện chưa tách riêng JD Manufacturing Engineering Manager; ENGM đang giữ cả cân bằng giữa DFM, process engineering và CAM release. | Nếu khối lượng NPI / clean / multi-axis tăng mạnh, cần tách thêm vai trò quản lý kỹ thuật chuyên sâu thay vì dồn mọi escalation vào ENGM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>D-ERP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ERP Administration Function</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Bo phan quan tri ERP</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>D-IT</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-epicor-handbook.html</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ESA</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Giữ Epicor vận hành như một hệ thống kiểm soát đáng tin cậy cho chuỗi RFQ → cash: đúng role, đúng workflow, đúng log thay đổi, đúng cấu hình và có khả năng hỗ trợ truy vết, kiểm toán và continuity khi có sự cố.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Dùng cho quyền hệ thống, workflow, cấu hình, change log và integrity giao dịch ERP; không dùng thay ESA trong phê duyệt cá nhân.</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD ERP Business Analyst hoặc Master Data Steward riêng; ESA đang giữ cả admin hệ thống lẫn nhiều phần việc phân tích / chuẩn hóa dữ liệu. | Nếu số lượng automation, integration hoặc report owner tăng mạnh, cần tách vai trò BA / data governance riêng để tránh dồn hết vào ESA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D-FIN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Finance Department</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Phong Tai chinh</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-finance-handbook.html</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>FIN, APAR, GLP</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Giữ độ tin cậy của tiền, chi phí và nghĩa vụ thanh toán trong doanh nghiệp job-order CNC: xuất hóa đơn đúng bằng chứng, theo dõi AR/AP rõ, nhìn được giá thành job và đóng sổ trên cơ sở dữ liệu có thể kiểm tra.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Dùng cho mandate tài chính và kiểm soát ghi nhận; không dùng thay FIN, APAR hoặc GLP trong quyết định cá nhân.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD Cost Accountant riêng; GLP và FIN đang cùng giữ job costing, variance review và month-end costing governance. | Nếu mức độ phức tạp của pricing / margin analysis tăng, cần tách vai trò cost controlling chuyên trách thay vì dồn vào team close hiện tại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>D-HR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Human Resources Department</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Phong Nhan su</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-hr-handbook.html</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Bảo đảm nguồn lực con người cho mô hình job-order CNC luôn sẵn sàng ở ba lớp: đủ người, đủ hồ sơ và đủ chứng nhận / training admin để D-PROD, D-ENG, D-QUAL, D-SCM, D-FIN, D-IT và D-EHS có thể xác nhận năng lực chuyên môn trên nền dữ liệu sạch.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Dùng cho workforce planning, hồ sơ nhân sự và điều phối đào tạo; sign-off năng lực chuyên môn vẫn phải quay về role quyết định thuộc D-PROD / D-ENG / D-QUAL / D-SCM / D-FIN / D-IT / D-EHS tùy công việc.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD Recruiter hoặc Training Coordinator riêng; HR đang giữ cả tuyển dụng và training administration dưới cùng một vai trò. | Nếu số lượng lao động, ca sản xuất hoặc apprenticeship program tăng, cần tách vai trò training / talent acquisition riêng để tránh quá tải hành chính.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>D-IT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>IT Department</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Phong CNTT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-it-handbook.html</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Bảo đảm hạ tầng số, tài khoản, backup và hỗ trợ người dùng luôn sẵn sàng, an toàn và truy được cho nhà máy job-order CNC, đồng thời làm rõ ranh giới giữa CNTT nền tảng với quản trị ERP và ownership dữ liệu nghiệp vụ.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>IT giữ nguyên viết tắt; dùng cho hạ tầng, endpoint, access, backup và support nền tảng.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD cybersecurity hoặc infrastructure engineer riêng; ITA đang giữ cả support, access control, baseline và một phần security hygiene. | Nếu external hosting, SIEM, zero-trust hoặc multi-site operations tăng lên, cần tách vai trò bảo mật / hạ tầng chuyên trách thay vì dồn vào ITA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>D-LOG</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Logistics and Shipping Function</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Bo phan Logistics va Giao van</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>LOG, SCM</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Dùng cho booking, shipment documents, carrier handoff và track-and-trace sau xuất hàng.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Dùng cho booking, shipment documents, carrier handoff và track-and-trace sau xuất hàng.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>D-PPC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Production Planning and Control Function</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Dieu do va kiem soat san xuat</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-production-handbook.html</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PPL, PD, WKM</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Dùng khi đang nói tới planning, dispatching và WIP control như một phân hệ ổn định thuộc D-PROD.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Dùng khi đang nói tới planning, dispatching và WIP control như một phân hệ ổn định thuộc D-PROD.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Production Department</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Phong San xuat</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-production-handbook.html</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PD, WKM, SL</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Biến kế hoạch và baseline kỹ thuật thành sản lượng thực tế an toàn, ổn định và truy được: đúng máy, đúng setup, đúng sequencing, đúng handoff và đúng dữ liệu hiện trường cho mô hình job-order CNC high-mix.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Dùng cho execution cấp xưởng; khi đi tới stop / restart / resource commitment phải truy về role code tương ứng.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD Maintenance Manager riêng; MNT đang giữ lớp kỹ thuật bảo trì thường nhật, còn ưu tiên máy và quyết định recovery cấp xưởng được PD / WKM giữ. | PIE đang gánh cả industrial engineering và một phần cải tiến hiện trường; nếu độ phức tạp layout / automation tăng cần tách vai trò chuyên sâu riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>D-PUR</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Purchasing Function</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Bo phan Mua hang</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>BUY, SCM</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Dùng cho sourcing, PO và supplier follow-up; không dùng thay BUY hoặc SCM khi đi tới cam kết với nhà cung cấp.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Dùng cho sourcing, PO và supplier follow-up; không dùng thay BUY hoặc SCM khi đi tới cam kết với nhà cung cấp.</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>D-QUAL</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Quality Department</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Phong Chat luong</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-quality-handbook.html</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>QA, QMS, QE, QCL, MCS</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Bảo vệ tính toàn vẹn của các cổng kiểm soát chất lượng từ incoming tới final release, giữ độ tin cậy của measurement system và biến sự cố chất lượng thành hành động ngăn tái diễn có bằng chứng.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Dùng cho mandate chất lượng cấp chức năng; các quyết định hold / release / disposition vẫn phải về role code.</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD Supplier Quality Engineer riêng; supplier quality escalation và SCAR đang do QA / QE phối hợp cùng SCM gánh. | Chưa có Internal Audit Lead full-time; QMS đang điều phối chương trình đánh giá với IAO hỗ trợ. Nếu tải audit tăng, cần tách vai trò chuyên trách.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Supply Chain Department</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Phong Chuoi cung ung</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>SCM, BUY, WAR, TOOL, LOG</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Bảo đảm nguyên vật liệu, dao cụ, outsource return, tồn kho, chứng từ và giao vận sẵn sàng đúng lúc, đúng trạng thái và truy được để nhà máy không dừng vì thiếu nguồn lực hoặc ship sai bằng chứng.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Dùng cho mô hình nguồn cung tổng thể; mua hàng, kho, tool crib và logistics là các phân hệ ổn định bên trong.</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD logistics supervisor riêng; D-LOG đang vận hành dưới khung quyết định của SCM. | Nếu supplier development hoặc outsource special process tăng mạnh, cần xem xét mở vai trò SQE / supplier development chuyên trách thay vì dồn vào QA và SCM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>D-SCS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Sales and Customer Service Department</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Phong Kinh doanh va Dich vu khach hang</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-sales-and-customer-service-handbook.html</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>CS, EST</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Biến nhu cầu của khách hàng thành cam kết nội bộ có kiểm soát: đúng scope, đúng revision, đúng giả định thương mại, đúng ngày giao có căn cứ và đúng tuyến phản hồi khi có thay đổi hoặc khiếu nại.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Dùng cho mandate cấp phòng ban; không dùng thay vai trò phê duyệt hoặc người giữ cam kết thương mại cá nhân.</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Hiện chưa có JD Commercial Manager hoặc Key Account Manager. Mọi cam kết vượt khung giá, điều khoản thanh toán, concession lớn hoặc account chiến lược hiện do CEO giữ. | Nếu tần suất deal ngoài chính sách hoặc số khách hàng chiến lược tăng, phải tách JD thương mại riêng thay vì tiếp tục dồn vào CS hoặc EST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>D-TCR</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tool Crib Function</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Bo phan Kho dao cu</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>TOOL, SCM</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Dùng cho quản lý dụng cụ cắt, preset, issue/return và tool life evidence.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Dùng cho quản lý dụng cụ cắt, preset, issue/return và tool life evidence.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>D-WHS</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Warehouse Function</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Bo phan Kho</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>WAR, SCM</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Dùng cho receiving, put-away, location control và inventory integrity.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Dùng cho receiving, put-away, location control và inventory integrity.</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add QMS Portal database foundation: schema, variable library, and technology report
- Add PostgreSQL 16+ database schema (103 tables, 121 enums, 140 indexes)
  with bitemporal audit trail, RLS, pgvector, partitioning
- Add variable_library.json V2 (1,061 variables, 53 categories)
  including global ERP variables from SAP/Oracle/Epicor/Dynamics
- Add database technology report (PostgreSQL + DuckDB + libSQL strategy)
- Update QMS docs, role boundaries, department handbooks, and core standards

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/data/qms-terminology-dictionary.xlsx
+++ b/tools/data/qms-terminology-dictionary.xlsx
@@ -539,7 +539,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>APAR | JD-APAR | Finance</t>
+          <t>APAR | JD-APAR | D-FIN</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BUY | JD-BUY | Supply Chain</t>
+          <t>BUY | JD-BUY | D-PUR, D-SCM</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CAM | JD-CAM | Engineering</t>
+          <t>CAM | JD-CAM | D-ENG</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CEO | JD-CEO | Executive</t>
+          <t>CEO | JD-CEO | D-EXEC</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CPS | JD-CPS | Production</t>
+          <t>CPS | JD-CPS | D-PROD</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CPT | JD-CPT | Production</t>
+          <t>CPT | JD-CPT | D-PROD</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CS | JD-CS | Sales</t>
+          <t>CS | JD-CS | D-SCS</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DBL | JD-DBL | Production</t>
+          <t>DBL | JD-DBL | D-PROD</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DBT | JD-DBT | Production</t>
+          <t>DBT | JD-DBT | D-PROD</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DFM | JD-DFM | Engineering</t>
+          <t>DFM | JD-DFM | D-ENG</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>EHS | JD-EHS | EHS</t>
+          <t>EHS | JD-EHS | D-EHS</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ENGM | JD-ENGM | Engineering</t>
+          <t>ENGM | JD-ENGM | D-ENG</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ESA | JD-ESA | IT</t>
+          <t>ESA | JD-ESA | D-ERP, D-IT</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EST | JD-EST | Sales</t>
+          <t>EST | JD-EST | D-SCS</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>FIN | JD-FIN | Finance</t>
+          <t>FIN | JD-FIN | D-FIN</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GLP | JD-GLP | Finance</t>
+          <t>GLP | JD-GLP | D-FIN</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>HR | JD-HR | HR</t>
+          <t>HR | JD-HR | D-HR</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>IAO | JD-IAO | Quality</t>
+          <t>IAO | JD-IAO | D-QUAL</t>
         </is>
       </c>
     </row>
@@ -989,7 +989,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ITA | JD-ITA | IT</t>
+          <t>ITA | JD-ITA | D-IT</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LOG | JD-LOG | Supply Chain</t>
+          <t>LOG | JD-LOG | D-LOG, D-SCM</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MCS | JD-MCS | Quality</t>
+          <t>MCS | JD-MCS | D-QUAL</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MNT | JD-MNT | Production</t>
+          <t>MNT | JD-MNT | D-PROD</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>OPR | JD-OPR | Production</t>
+          <t>OPR | JD-OPR | D-PROD</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>PD | JD-PD | Production</t>
+          <t>PD | JD-PD | D-PROD</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PE | JD-PE | Engineering</t>
+          <t>PE | JD-PE | D-ENG</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PIE | JD-PIE | Production</t>
+          <t>PIE | JD-PIE | D-PROD</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>PPL | JD-PPL | Production</t>
+          <t>PPL | JD-PPL | D-PPC, D-PROD</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>QA | JD-QA | Quality</t>
+          <t>QA | JD-QA | D-QUAL</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>QC | JD-QC | Quality</t>
+          <t>QC | JD-QC | D-QUAL</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>QCL | JD-QCL | Quality</t>
+          <t>QCL | JD-QCL | D-QUAL</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>QE | JD-QE | Quality</t>
+          <t>QE | JD-QE | D-QUAL</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>QMS | JD-QMS | Quality</t>
+          <t>QMS | JD-QMS | D-QUAL</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SCM | JD-SCM | Supply Chain</t>
+          <t>SCM | JD-SCM | D-SCM</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SET | JD-SET | Production</t>
+          <t>SET | JD-SET | D-PROD</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SL | JD-SL | Production</t>
+          <t>SL | JD-SL | D-PROD</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>TOOL | JD-TOOL | Supply Chain</t>
+          <t>TOOL | JD-TOOL | D-TCR, D-SCM</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>WAR | JD-WAR | Supply Chain</t>
+          <t>WAR | JD-WAR | D-WHS, D-SCM</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>WKM | JD-WKM | Production</t>
+          <t>WKM | JD-WKM | D-PROD</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4848,12 +4848,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sales and Customer Service Department</t>
+          <t>Executive Department</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Phòng Kinh doanh và Dịch vụ khách hàng</t>
+          <t>Phòng Điều hành</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4863,7 +4863,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dùng cho mandate cấp phòng ban; không dùng thay vai trò phê duyệt hoặc người giữ cam kết thương mại cá nhân.</t>
+          <t>Dùng cho lớp điều hành cấp doanh nghiệp; chỉ dùng khi đang nói tới mandate cấp điều hành hoặc enterprise-level resource steering, không dùng thay vai trò quyết định cá nhân của CEO.</t>
         </is>
       </c>
     </row>
@@ -4873,12 +4873,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Engineering Department</t>
+          <t>Sales and Customer Service Department</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Phòng Kỹ thuật</t>
+          <t>Phòng Kinh doanh và Dịch vụ khách hàng</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4888,7 +4888,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Dùng cho thiết kế công nghệ, baseline và release cấp chức năng; không dùng thay ENGM, DFM, PE hoặc CAM trong ô quyết định.</t>
+          <t>Dùng cho mandate cấp phòng ban; không dùng thay vai trò phê duyệt hoặc người giữ cam kết thương mại cá nhân.</t>
         </is>
       </c>
     </row>
@@ -4898,12 +4898,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Production Department</t>
+          <t>Engineering Department</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Phòng Sản xuất</t>
+          <t>Phòng Kỹ thuật</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -4913,7 +4913,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Dùng cho execution cấp xưởng; khi đi tới stop / restart / resource commitment phải truy về role code tương ứng.</t>
+          <t>Dùng cho thiết kế công nghệ, baseline và release cấp chức năng; không dùng thay ENGM, DFM, PE hoặc CAM trong ô quyết định.</t>
         </is>
       </c>
     </row>
@@ -4923,12 +4923,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Production Planning and Control Function</t>
+          <t>Production Department</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Phân hệ Điều độ và Kiểm soát sản xuất</t>
+          <t>Phòng Sản xuất</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dùng khi đang nói tới planning, dispatching và WIP control như một phân hệ ổn định thuộc D-PROD.</t>
+          <t>Dùng cho execution cấp xưởng; khi đi tới stop / restart / resource commitment phải truy về role code tương ứng.</t>
         </is>
       </c>
     </row>
@@ -4948,12 +4948,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Quality Department</t>
+          <t>Production Planning and Control Function</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Phòng Chất lượng</t>
+          <t>Phân hệ Điều độ và Kiểm soát sản xuất</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dùng cho mandate chất lượng cấp chức năng; các quyết định hold / release / disposition vẫn phải về role code.</t>
+          <t>Dùng khi đang nói tới planning, dispatching và WIP control như một phân hệ ổn định thuộc D-PROD.</t>
         </is>
       </c>
     </row>
@@ -4973,12 +4973,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Supply Chain Department</t>
+          <t>Quality Department</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Phòng Chuỗi cung ứng</t>
+          <t>Phòng Chất lượng</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4988,7 +4988,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Dùng cho mô hình nguồn cung tổng thể; mua hàng, kho, tool crib và logistics là các phân hệ ổn định bên trong.</t>
+          <t>Dùng cho mandate chất lượng cấp chức năng; các quyết định hold / release / disposition vẫn phải về role code.</t>
         </is>
       </c>
     </row>
@@ -4998,12 +4998,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Purchasing Function</t>
+          <t>Supply Chain Department</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Phân hệ Mua hàng</t>
+          <t>Phòng Chuỗi cung ứng</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dùng cho sourcing, PO và supplier follow-up; không dùng thay BUY hoặc SCM khi đi tới cam kết với nhà cung cấp.</t>
+          <t>Dùng cho mô hình nguồn cung tổng thể; mua hàng, kho, tool crib và logistics là các phân hệ ổn định bên trong.</t>
         </is>
       </c>
     </row>
@@ -5023,12 +5023,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Warehouse Function</t>
+          <t>Purchasing Function</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Phân hệ Kho</t>
+          <t>Phân hệ Mua hàng</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Dùng cho receiving, put-away, location control và inventory integrity.</t>
+          <t>Dùng cho sourcing, PO và supplier follow-up; không dùng thay BUY hoặc SCM khi đi tới cam kết với nhà cung cấp.</t>
         </is>
       </c>
     </row>
@@ -5048,12 +5048,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tool Crib Function</t>
+          <t>Warehouse Function</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Phân hệ Kho dao cụ</t>
+          <t>Phân hệ Kho</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Dùng cho quản lý dụng cụ cắt, preset, issue/return và tool life evidence.</t>
+          <t>Dùng cho receiving, put-away, location control và inventory integrity.</t>
         </is>
       </c>
     </row>
@@ -5073,12 +5073,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Logistics and Shipping Function</t>
+          <t>Tool Crib Function</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Phân hệ Logistics và Giao vận</t>
+          <t>Phân hệ Kho dao cụ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Dùng cho booking, shipment documents, carrier handoff và track-and-trace sau xuất hàng.</t>
+          <t>Dùng cho quản lý dụng cụ cắt, preset, issue/return và tool life evidence.</t>
         </is>
       </c>
     </row>
@@ -5098,12 +5098,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Finance Department</t>
+          <t>Logistics and Shipping Function</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Phòng Tài chính</t>
+          <t>Phân hệ Logistics và Giao vận</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Dùng cho mandate tài chính và kiểm soát ghi nhận; không dùng thay FIN, APAR hoặc GLP trong quyết định cá nhân.</t>
+          <t>Dùng cho booking, shipment documents, carrier handoff và track-and-trace sau xuất hàng.</t>
         </is>
       </c>
     </row>
@@ -5123,12 +5123,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Human Resources Department</t>
+          <t>Finance Department</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Phòng Nhân sự</t>
+          <t>Phòng Tài chính</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Dùng cho workforce planning, hồ sơ nhân sự và điều phối đào tạo; sign-off năng lực chuyên môn vẫn phải quay về role quyết định thuộc D-PROD / D-ENG / D-QUAL / D-SCM / D-FIN / D-IT / D-EHS tùy công việc.</t>
+          <t>Dùng cho mandate tài chính và kiểm soát ghi nhận; không dùng thay FIN, APAR hoặc GLP trong quyết định cá nhân.</t>
         </is>
       </c>
     </row>
@@ -5148,12 +5148,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EHS Department</t>
+          <t>Human Resources Department</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Phòng EHS</t>
+          <t>Phòng Nhân sự</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>EHS giữ nguyên viết tắt; dùng cho mandate an toàn, môi trường và emergency preparedness.</t>
+          <t>Dùng cho workforce planning, hồ sơ nhân sự và điều phối đào tạo; sign-off năng lực chuyên môn vẫn phải quay về role quyết định thuộc D-PROD / D-ENG / D-QUAL / D-SCM / D-FIN / D-IT / D-EHS tùy công việc.</t>
         </is>
       </c>
     </row>
@@ -5173,12 +5173,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IT Department</t>
+          <t>EHS Department</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Phòng CNTT</t>
+          <t>Phòng EHS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -5188,7 +5188,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>IT giữ nguyên viết tắt; dùng cho hạ tầng, endpoint, access, backup và support nền tảng.</t>
+          <t>EHS giữ nguyên viết tắt; dùng cho mandate an toàn, môi trường và emergency preparedness.</t>
         </is>
       </c>
     </row>
@@ -5198,12 +5198,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ERP Administration Function</t>
+          <t>IT Department</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Phân hệ Quản trị ERP</t>
+          <t>Phòng CNTT</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Dùng cho quyền hệ thống, workflow, cấu hình, change log và integrity giao dịch ERP; không dùng thay ESA trong phê duyệt cá nhân.</t>
+          <t>IT giữ nguyên viết tắt; dùng cho hạ tầng, endpoint, access, backup và support nền tảng.</t>
         </is>
       </c>
     </row>
@@ -5223,12 +5223,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Department coverage gap</t>
+          <t>ERP Administration Function</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Khoảng trống bao phủ phòng ban</t>
+          <t>Phân hệ Quản trị ERP</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Dùng khi công việc có thật nhưng handbook hoặc department code chưa bao phủ rõ.</t>
+          <t>Dùng cho quyền hệ thống, workflow, cấu hình, change log và integrity giao dịch ERP; không dùng thay ESA trong phê duyệt cá nhân.</t>
         </is>
       </c>
     </row>
@@ -5248,12 +5248,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Subfunction coverage gap</t>
+          <t>Department coverage gap</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Khoảng trống bao phủ phân hệ</t>
+          <t>Khoảng trống bao phủ phòng ban</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -5263,7 +5263,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Dùng khi cần tách một phân hệ ổn định lặp lại nhưng hệ thống chưa khai báo D-code tương ứng.</t>
+          <t>Dùng khi công việc có thật nhưng handbook hoặc department code chưa bao phủ rõ.</t>
         </is>
       </c>
     </row>
@@ -5273,20 +5273,45 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>Subfunction coverage gap</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Khoảng trống bao phủ phân hệ</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Dùng khi cần tách một phân hệ ổn định lặp lại nhưng hệ thống chưa khai báo D-code tương ứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>JD gap</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Khoảng trống chức danh gắn JD</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>Dùng khi công việc đi tới quyết định cá nhân nhưng hệ thống chưa có JD tương ứng; không được che bằng tên phòng ban.</t>
         </is>
@@ -5675,7 +5700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5701,20 +5726,35 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Phong ban</t>
+          <t>Legacy department label</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Department codes</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Reports to role code</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Direct reports role codes</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>JD code</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>JD path</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Governance hats</t>
         </is>
@@ -5746,14 +5786,26 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>D-FIN</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FIN</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>JD-APAR</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/07-JD-Finance/jd-ap-ar-and-payments-accountant.html</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -5781,14 +5833,26 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>D-PUR, D-SCM</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SCM</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>JD-BUY</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-buyer-purchasing.html</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -5816,14 +5880,26 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>D-ENG</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ENGM</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>JD-CAM</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/03-JD-Engineering/jd-cam-nc-programmer.html</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -5846,20 +5922,31 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Executive</t>
+          <t>Executive Department</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>D-EXEC</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PD, QA, SCM, FIN, HR, EHS, ITA, CS, EST</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>JD-CEO</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/01-JD-Executive/jd-chief-executive-officer.html</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>IC-BIZ</t>
         </is>
@@ -5891,14 +5978,30 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CPT</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>JD-CPS</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-cleaning-and-packaging-supervisor.html</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -5926,14 +6029,26 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CPS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>JD-CPT</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-cleaning-packaging-technician.html</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -5961,14 +6076,26 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>D-SCS</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>JD-CS</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/06-JD-Sales/jd-customer-service.html</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -5996,14 +6123,30 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>WKM</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>DBT</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>JD-DBL</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-deburr-team-lead.html</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -6031,14 +6174,26 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>DBL</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>JD-DBT</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-deburr-technician.html</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -6066,14 +6221,26 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>D-ENG</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ENGM</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>JD-DFM</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/03-JD-Engineering/jd-dfm-engineer.html</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -6101,15 +6268,26 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>D-EHS</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
           <t>JD-EHS</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/09-JD-EHS/jd-ehs-specialist.html</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>IC-EHS</t>
         </is>
@@ -6141,14 +6319,30 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>D-ENG</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>DFM, PE, CAM</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
           <t>JD-ENGM</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/03-JD-Engineering/jd-engineering-lead-manager.html</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -6176,15 +6370,26 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>D-ERP, D-IT</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
           <t>JD-ESA</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/10-JD-IT/jd-epicor-system-administrator.html</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>IC-IT</t>
         </is>
@@ -6216,14 +6421,26 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>D-SCS</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
           <t>JD-EST</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/06-JD-Sales/jd-estimator.html</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -6251,14 +6468,30 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>D-FIN</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>APAR, GLP</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>JD-FIN</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/07-JD-Finance/jd-finance-manager.html</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -6286,14 +6519,26 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>D-FIN</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>FIN</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
           <t>JD-GLP</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/07-JD-Finance/jd-general-ledger-and-payroll-accountant.html</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -6321,14 +6566,26 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>D-HR</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
           <t>JD-HR</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/08-JD-HR/jd-hr-manager.html</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -6356,14 +6613,26 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>D-QUAL</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>JD-IAO</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-internal-auditor-outsource.html</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -6391,15 +6660,30 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>D-IT</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ESA</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>JD-ITA</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/10-JD-IT/jd-it-admin.html</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>IC-IT</t>
         </is>
@@ -6431,14 +6715,26 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>D-LOG, D-SCM</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>SCM</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>JD-LOG</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-logistics-shipping-coordinator.html</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -6466,14 +6762,26 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>D-QUAL</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
           <t>JD-MCS</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-metrology-and-calibration-specialist.html</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -6501,14 +6809,26 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>JD-MNT</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-maintenance-technician.html</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -6536,14 +6856,26 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
           <t>JD-OPR</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-cnc-operator.html</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -6571,15 +6903,30 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ENGM, PPL, WKM, CPS, MNT, PIE</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
           <t>JD-PD</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/01-JD-Executive/jd-production-director.html</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>IC-PROD</t>
         </is>
@@ -6611,14 +6958,26 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
+          <t>D-ENG</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>ENGM</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
           <t>JD-PE</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/03-JD-Engineering/jd-process-engineer.html</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -6646,15 +7005,26 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>JD-PIE</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-production-engineer-industrial-engineer.html</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>CI</t>
         </is>
@@ -6686,14 +7056,26 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
+          <t>D-PPC, D-PROD</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
           <t>JD-PPL</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-production-planner.html</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -6721,15 +7103,30 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
+          <t>D-QUAL</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>QMS, QE, QCL, MCS, IAO</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
           <t>JD-QA</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-qa-manager.html</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>QMR, PSO</t>
         </is>
@@ -6761,14 +7158,26 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
+          <t>D-QUAL</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>QCL</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
           <t>JD-QC</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-qc-inspector-cmm-programmer-operator.html</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -6796,14 +7205,30 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
+          <t>D-QUAL</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
           <t>JD-QCL</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-qc-inspector-lead.html</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -6831,14 +7256,26 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
+          <t>D-QUAL</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>JD-QE</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-quality-engineer.html</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -6866,15 +7303,26 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
+          <t>D-QUAL</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
           <t>JD-QMS</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/04-JD-Quality/jd-qms-engineer.html</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>DC, LA</t>
         </is>
@@ -6906,14 +7354,30 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
+          <t>D-SCM</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>BUY, WAR, TOOL, LOG</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
           <t>JD-SCM</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-supply-chain-manager.html</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -6941,14 +7405,26 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>WKM</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
           <t>JD-SET</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-setup-technician.html</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -6976,14 +7452,30 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>WKM</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>OPR</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
           <t>JD-SL</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-shift-leader.html</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -7011,14 +7503,26 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
+          <t>D-TCR, D-SCM</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>SCM</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
           <t>JD-TOOL</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-tool-crib-tool-storekeeper.html</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -7046,14 +7550,26 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
+          <t>D-WHS, D-SCM</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>SCM</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
           <t>JD-WAR</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/05-JD-Supply-Chain/jd-warehouse-clerk.html</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -7081,14 +7597,30 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
+          <t>D-PROD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>SL, SET, DBL</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
           <t>JD-WKM</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/03-Job-Descriptions/02-JD-Production/jd-cnc-workshop-manager.html</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7367,7 +7899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7388,12 +7920,12 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Tên tiếng Việt chuẩn</t>
+          <t>Ten tieng Viet chuan</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Loại</t>
+          <t>Loai</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -7409,21 +7941,6 @@
       <c r="H1" t="inlineStr">
         <is>
           <t>Lead roles</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Mandate summary</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Boundary / use note</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Coverage gap / expansion trigger</t>
         </is>
       </c>
     </row>
@@ -7461,21 +7978,6 @@
           <t>EHS</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Bảo vệ con người, môi trường làm việc và tài sản vận hành bằng một hệ thống an toàn thực chiến: nhận diện mối nguy, giữ kỷ luật permit / LOTO, điều tra học từ sự cố và duy trì readiness cho tình huống khẩn cấp trong nhà máy job-order CNC.</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>EHS giữ nguyên viết tắt; dùng cho mandate an toàn, môi trường và emergency preparedness.</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD EHS Manager; EHS Specialist đang giữ phương pháp và điều phối chính, còn quyết định plant-wide shutdown hoặc reopening vẫn do CEO / PD giữ. | Nếu nhà máy mở thêm hoạt động rủi ro cao hoặc tăng tải compliance / contractor, cần xem xét mở vai trò quản lý EHS riêng thay vì giữ một chuyên viên đơn tuyến.</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -7511,21 +8013,6 @@
           <t>ENGM, DFM, PE, CAM</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Biến yêu cầu kỹ thuật của khách hàng thành baseline gia công đáng tin cậy: đúng process, đúng chương trình, đúng control requirement và đủ dữ liệu để production, quality và planning có thể thực thi mà không phải suy diễn.</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Dùng cho thiết kế công nghệ, baseline và release cấp chức năng; không dùng thay ENGM, DFM, PE hoặc CAM trong ô quyết định.</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Hiện chưa tách riêng JD Manufacturing Engineering Manager; ENGM đang giữ cả cân bằng giữa DFM, process engineering và CAM release. | Nếu khối lượng NPI / clean / multi-axis tăng mạnh, cần tách thêm vai trò quản lý kỹ thuật chuyên sâu thay vì dồn mọi escalation vào ENGM.</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -7566,21 +8053,6 @@
           <t>ESA</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Giữ Epicor vận hành như một hệ thống kiểm soát đáng tin cậy cho chuỗi RFQ → cash: đúng role, đúng workflow, đúng log thay đổi, đúng cấu hình và có khả năng hỗ trợ truy vết, kiểm toán và continuity khi có sự cố.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Dùng cho quyền hệ thống, workflow, cấu hình, change log và integrity giao dịch ERP; không dùng thay ESA trong phê duyệt cá nhân.</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD ERP Business Analyst hoặc Master Data Steward riêng; ESA đang giữ cả admin hệ thống lẫn nhiều phần việc phân tích / chuẩn hóa dữ liệu. | Nếu số lượng automation, integration hoặc report owner tăng mạnh, cần tách vai trò BA / data governance riêng để tránh dồn hết vào ESA.</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -7588,17 +8060,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>D-FIN</t>
+          <t>D-EXEC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Finance Department</t>
+          <t>Executive Department</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Phong Tai chinh</t>
+          <t>Phong Dieu hanh</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7608,27 +8080,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-finance-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-executive-handbook.html</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>FIN, APAR, GLP</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Giữ độ tin cậy của tiền, chi phí và nghĩa vụ thanh toán trong doanh nghiệp job-order CNC: xuất hóa đơn đúng bằng chứng, theo dõi AR/AP rõ, nhìn được giá thành job và đóng sổ trên cơ sở dữ liệu có thể kiểm tra.</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Dùng cho mandate tài chính và kiểm soát ghi nhận; không dùng thay FIN, APAR hoặc GLP trong quyết định cá nhân.</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD Cost Accountant riêng; GLP và FIN đang cùng giữ job costing, variance review và month-end costing governance. | Nếu mức độ phức tạp của pricing / margin analysis tăng, cần tách vai trò cost controlling chuyên trách thay vì dồn vào team close hiện tại.</t>
+          <t>CEO</t>
         </is>
       </c>
     </row>
@@ -7638,17 +8095,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>D-HR</t>
+          <t>D-FIN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Human Resources Department</t>
+          <t>Finance Department</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Phong Nhan su</t>
+          <t>Phong Tai chinh</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -7658,27 +8115,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-hr-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-finance-handbook.html</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Bảo đảm nguồn lực con người cho mô hình job-order CNC luôn sẵn sàng ở ba lớp: đủ người, đủ hồ sơ và đủ chứng nhận / training admin để D-PROD, D-ENG, D-QUAL, D-SCM, D-FIN, D-IT và D-EHS có thể xác nhận năng lực chuyên môn trên nền dữ liệu sạch.</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Dùng cho workforce planning, hồ sơ nhân sự và điều phối đào tạo; sign-off năng lực chuyên môn vẫn phải quay về role quyết định thuộc D-PROD / D-ENG / D-QUAL / D-SCM / D-FIN / D-IT / D-EHS tùy công việc.</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD Recruiter hoặc Training Coordinator riêng; HR đang giữ cả tuyển dụng và training administration dưới cùng một vai trò. | Nếu số lượng lao động, ca sản xuất hoặc apprenticeship program tăng, cần tách vai trò training / talent acquisition riêng để tránh quá tải hành chính.</t>
+          <t>FIN, APAR, GLP</t>
         </is>
       </c>
     </row>
@@ -7688,17 +8130,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>D-IT</t>
+          <t>D-HR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>IT Department</t>
+          <t>Human Resources Department</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Phong CNTT</t>
+          <t>Phong Nhan su</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -7708,27 +8150,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-it-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-hr-handbook.html</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>ITA</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Bảo đảm hạ tầng số, tài khoản, backup và hỗ trợ người dùng luôn sẵn sàng, an toàn và truy được cho nhà máy job-order CNC, đồng thời làm rõ ranh giới giữa CNTT nền tảng với quản trị ERP và ownership dữ liệu nghiệp vụ.</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>IT giữ nguyên viết tắt; dùng cho hạ tầng, endpoint, access, backup và support nền tảng.</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD cybersecurity hoặc infrastructure engineer riêng; ITA đang giữ cả support, access control, baseline và một phần security hygiene. | Nếu external hosting, SIEM, zero-trust hoặc multi-site operations tăng lên, cần tách vai trò bảo mật / hạ tầng chuyên trách thay vì dồn vào ITA.</t>
+          <t>HR</t>
         </is>
       </c>
     </row>
@@ -7738,50 +8165,34 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>D-LOG</t>
+          <t>D-IT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Logistics and Shipping Function</t>
+          <t>IT Department</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Bo phan Logistics va Giao van</t>
+          <t>Phong CNTT</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>subfunction</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>D-SCM</t>
+          <t>department</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-it-handbook.html</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>LOG, SCM</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Dùng cho booking, shipment documents, carrier handoff và track-and-trace sau xuất hàng.</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Dùng cho booking, shipment documents, carrier handoff và track-and-trace sau xuất hàng.</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
+          <t>ITA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -7789,17 +8200,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>D-PPC</t>
+          <t>D-LOG</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Production Planning and Control Function</t>
+          <t>Logistics and Shipping Function</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Dieu do va kiem soat san xuat</t>
+          <t>Bo phan Logistics va Giao van</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -7809,30 +8220,19 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>D-PROD</t>
+          <t>D-SCM</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-production-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>PPL, PD, WKM</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Dùng khi đang nói tới planning, dispatching và WIP control như một phân hệ ổn định thuộc D-PROD.</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Dùng khi đang nói tới planning, dispatching và WIP control như một phân hệ ổn định thuộc D-PROD.</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr"/>
+          <t>LOG, SCM</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -7840,24 +8240,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>D-PPC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Production Planning and Control Function</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Dieu do va kiem soat san xuat</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>D-PROD</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Production Department</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Phong San xuat</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>department</t>
-        </is>
-      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-production-handbook.html</t>
@@ -7865,22 +8270,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>PD, WKM, SL</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Biến kế hoạch và baseline kỹ thuật thành sản lượng thực tế an toàn, ổn định và truy được: đúng máy, đúng setup, đúng sequencing, đúng handoff và đúng dữ liệu hiện trường cho mô hình job-order CNC high-mix.</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Dùng cho execution cấp xưởng; khi đi tới stop / restart / resource commitment phải truy về role code tương ứng.</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD Maintenance Manager riêng; MNT đang giữ lớp kỹ thuật bảo trì thường nhật, còn ưu tiên máy và quyết định recovery cấp xưởng được PD / WKM giữ. | PIE đang gánh cả industrial engineering và một phần cải tiến hiện trường; nếu độ phức tạp layout / automation tăng cần tách vai trò chuyên sâu riêng.</t>
+          <t>PPL, PD, WKM</t>
         </is>
       </c>
     </row>
@@ -7890,50 +8280,34 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>D-PUR</t>
+          <t>D-PROD</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Purchasing Function</t>
+          <t>Production Department</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bo phan Mua hang</t>
+          <t>Phong San xuat</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>subfunction</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>D-SCM</t>
+          <t>department</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-production-handbook.html</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>BUY, SCM</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Dùng cho sourcing, PO và supplier follow-up; không dùng thay BUY hoặc SCM khi đi tới cam kết với nhà cung cấp.</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Dùng cho sourcing, PO và supplier follow-up; không dùng thay BUY hoặc SCM khi đi tới cam kết với nhà cung cấp.</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
+          <t>PD, WKM, SL</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -7941,47 +8315,37 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>D-QUAL</t>
+          <t>D-PUR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Quality Department</t>
+          <t>Purchasing Function</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Phong Chat luong</t>
+          <t>Bo phan Mua hang</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>department</t>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-quality-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>QA, QMS, QE, QCL, MCS</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Bảo vệ tính toàn vẹn của các cổng kiểm soát chất lượng từ incoming tới final release, giữ độ tin cậy của measurement system và biến sự cố chất lượng thành hành động ngăn tái diễn có bằng chứng.</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Dùng cho mandate chất lượng cấp chức năng; các quyết định hold / release / disposition vẫn phải về role code.</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD Supplier Quality Engineer riêng; supplier quality escalation và SCAR đang do QA / QE phối hợp cùng SCM gánh. | Chưa có Internal Audit Lead full-time; QMS đang điều phối chương trình đánh giá với IAO hỗ trợ. Nếu tải audit tăng, cần tách vai trò chuyên trách.</t>
+          <t>BUY, SCM</t>
         </is>
       </c>
     </row>
@@ -7991,17 +8355,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>D-SCM</t>
+          <t>D-QUAL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Supply Chain Department</t>
+          <t>Quality Department</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Phong Chuoi cung ung</t>
+          <t>Phong Chat luong</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -8011,27 +8375,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-quality-handbook.html</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SCM, BUY, WAR, TOOL, LOG</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Bảo đảm nguyên vật liệu, dao cụ, outsource return, tồn kho, chứng từ và giao vận sẵn sàng đúng lúc, đúng trạng thái và truy được để nhà máy không dừng vì thiếu nguồn lực hoặc ship sai bằng chứng.</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Dùng cho mô hình nguồn cung tổng thể; mua hàng, kho, tool crib và logistics là các phân hệ ổn định bên trong.</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD logistics supervisor riêng; D-LOG đang vận hành dưới khung quyết định của SCM. | Nếu supplier development hoặc outsource special process tăng mạnh, cần xem xét mở vai trò SQE / supplier development chuyên trách thay vì dồn vào QA và SCM.</t>
+          <t>QA, QMS, QE, QCL, MCS</t>
         </is>
       </c>
     </row>
@@ -8041,17 +8390,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>D-SCS</t>
+          <t>D-SCM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sales and Customer Service Department</t>
+          <t>Supply Chain Department</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Phong Kinh doanh va Dich vu khach hang</t>
+          <t>Phong Chuoi cung ung</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -8061,27 +8410,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-sales-and-customer-service-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CS, EST</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Biến nhu cầu của khách hàng thành cam kết nội bộ có kiểm soát: đúng scope, đúng revision, đúng giả định thương mại, đúng ngày giao có căn cứ và đúng tuyến phản hồi khi có thay đổi hoặc khiếu nại.</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Dùng cho mandate cấp phòng ban; không dùng thay vai trò phê duyệt hoặc người giữ cam kết thương mại cá nhân.</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Hiện chưa có JD Commercial Manager hoặc Key Account Manager. Mọi cam kết vượt khung giá, điều khoản thanh toán, concession lớn hoặc account chiến lược hiện do CEO giữ. | Nếu tần suất deal ngoài chính sách hoặc số khách hàng chiến lược tăng, phải tách JD thương mại riêng thay vì tiếp tục dồn vào CS hoặc EST.</t>
+          <t>SCM, BUY, WAR, TOOL, LOG</t>
         </is>
       </c>
     </row>
@@ -8091,50 +8425,34 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>D-TCR</t>
+          <t>D-SCS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tool Crib Function</t>
+          <t>Sales and Customer Service Department</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bo phan Kho dao cu</t>
+          <t>Phong Kinh doanh va Dich vu khach hang</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>subfunction</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>D-SCM</t>
+          <t>department</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-sales-and-customer-service-handbook.html</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TOOL, SCM</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Dùng cho quản lý dụng cụ cắt, preset, issue/return và tool life evidence.</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Dùng cho quản lý dụng cụ cắt, preset, issue/return và tool life evidence.</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
+          <t>CS, EST</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -8142,50 +8460,79 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>D-TCR</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Tool Crib Function</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Bo phan Kho dao cu</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>TOOL, SCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>D-WHS</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Warehouse Function</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Bo phan Kho</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>subfunction</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>D-SCM</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>WAR, SCM</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Dùng cho receiving, put-away, location control và inventory integrity.</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Dùng cho receiving, put-away, location control và inventory integrity.</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Overhaul forms portal and refresh QMS operations documentation
</commit_message>
<xml_diff>
--- a/tools/data/qms-terminology-dictionary.xlsx
+++ b/tools/data/qms-terminology-dictionary.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role code &amp; JD link" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance hats" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Department code &amp; handbook link" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bundle glossary" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vai tro &amp; Chuc danh'!$A$1:$E$37</definedName>
@@ -1474,6 +1475,967 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Bundle code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Label English</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Ten / dien giai tieng Viet</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Loai</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Thanh phan</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Duoc dung khi</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Khong dung de che</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Glossary path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ALL_DEPTS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>All Departments</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Toan bo phong ban va phan he da cong bo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>department bundle</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>D-SCS, D-ENG, D-PROD, D-PPC, D-MNT, D-QUAL, D-SCM, D-PUR, D-WHS, D-TCR, D-LOG, D-FIN, D-HR, D-EHS, D-IT, D-ERP</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Dung khi tai lieu dang noi toi pham vi bao phu toan doanh nghiep o muc mandate cap phong ban.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Khong dung cho phe duyet, hold/release hoac named accountability.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AREA_LEADS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Area Leads</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Nhom dau moi khu vuc hien truong</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SL, WKM, CPS, QCL</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Dung cho lop dau moi kiem soat theo khu vuc / khu thao tac tren san xuat.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Khong dung de thay direct line manager hay func head khi dang noi toi authority cap cao hon.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>COMMERCIAL_FRONT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Commercial Front</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nhom dau moi thuong mai</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CS, EST</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Dung cho lop dau moi tiep nhan RFQ, xu ly thuong mai va dieu kien don hang.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Khong dung thay CEO khi tai lieu dang noi toi commitment vuot khung.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DATA_OWNERS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Business Data Owners</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Nhom so huu du lieu nghiep vu</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CS, EST, PD, ENGM, QA[QMR], SCM, FIN, HR, EHS, ITA</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Dung khi tai lieu dang noi toi lop actor so huu du lieu nghiep vu, KPI, cau hinh giao dich hoac quy tac nghiep vu theo chuc nang.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Khong dung de thay owner he thong ky thuat, admin nen tang hay role phe duyet cu the.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DEPLOYMENT_LEADS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Deployment Leads</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Nhom dau moi trien khai theo ca va phong ban</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>WKM, SL, DBL, CPS, QCL, HR</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Dung cho nhom champion / lead thuc thi rollout, training, adoption va go-live tai hien truong.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Khong dung de thay deployment steering group hoac owner KPI/MR.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DEPLOYMENT_STEERING</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Deployment Steering Group</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Nhom chi dao trien khai lien chuc nang</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>CEO, PD, ENGM, QA[QMR], SCM, FIN, HR, EHS, ITA</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Dung cho nhom chi dao go-live, cutover, deployment va dong bo lien phong ban.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Khong dung de thay tung owner thuc thi, champion hay direct line manager tai hien truong.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DIRECT_LINE_MGRS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Direct Line Managers</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Nhom quan ly truc tiep</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CEO, PD, ENGM, QA[QMR], SCM, FIN, HR, EHS, ITA, WKM, SL, DBL, CPS, QCL</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Dung khi dang noi toi layer quan ly truc tiep phan cong, danh gia, backup activation va theo doi nang luc.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Khong dung de thay func heads khi tai lieu dang noi toi authority cap phong ban.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ENG_RELEASE_CORE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Engineering Release Core</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Nhom nong cot phat hanh ky thuat</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ENGM, DFM, PE, CAM</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Dung cho lop role phoi hop DFM, process planning va program release.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Khong dung de thay ENGM neu tai lieu dang noi toi owner phat hanh ky thuat.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FRONTLINE_LEADS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Frontline Leads</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Nhom dieu hanh tuyen dau</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>WKM, SL, DBL, CPS, QCL</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Dung cho cac role lead / supervisor truc tiep kiem thuc thi tai xuong, tai diem dung hoac tai khu phu tro.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Khong dung de thay lead cap chuc nang hay phe duyet cap phong ban.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FUNC_HEADS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Function Heads</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Nhom dau moi dieu hanh chuc nang</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PD, ENGM, QA[QMR], SCM, FIN, HR, EHS, ITA</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Dung khi tai lieu dang noi toi lop dau moi dieu hanh cap chuc nang cua cac khoi chinh.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Khong dung thay nguoi phe duyet cu the neu da xac dinh duoc role ra quyet dinh.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>FUNC_OWNERS</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Functional Content Owners</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Nhom so huu noi dung nghiep vu theo chuc nang</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CS, EST, PD, ENGM, QA[QMR], SCM, FIN, HR, EHS, ITA</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Dung khi can goi ten lop actor so huu noi dung nghiep vu cua du lieu, KPI hoac quy tac giao dich.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Khong dung de che mo ranh gioi giua owner du lieu nghiep vu va role ky thuat he thong.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE_SMES</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Knowledge SMEs</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Nhom chuyen gia tri thuc</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>DFM, CAM, PE, QE, MCS, WKM, SET, QCL, MNT, TOOL, ESA</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Dung cho nhom role giu tri thuc chuyen sau can chuyen giao, chuan hoa va tai su dung.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Khong dung thay func owner hoac direct line manager trong quyet dinh nhan su.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MR_REPORT_OWNERS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Management Review Report Owners</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Nhom chu tri goi bao cao MR va KPI</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>CS, EST, PD, ENGM, QA[QMR], QMS, SCM, FIN, HR, EHS, ITA</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Dung cho lop role chot, nop va giai trinh goi bao cao KPI / MR.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Khong dung de thay role xac nhan nguon du lieu hoac ITA / ESA.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>OJT_COACHES</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>OJT Coaches</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Nhom huan luyen OJT</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ENGM, PE, QE, MCS, WKM, SL, SET, QCL, MNT, TOOL, ESA</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Dung cho lop actor duoc giao kem cap, huong dan thao tac va danh gia OJT theo pham vi duoc phe duyet.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Khong dung de thay named evaluator neu tai lieu da chi ro ro ai la nguoi danh gia.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>OPS_SCOPE_OWNERS</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Operational Scope Owners</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Nhom dau moi so huu pham vi van hanh</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CS, EST, PPL, PD, ENGM, QA[QMR], QMS, SCM, FIN, HR, EHS, ITA, WKM, SL, QCL, LOG</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Dung cho lop actor so huu pham vi van hanh giao nhau giua nhieu chuc nang trong job-order CNC.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Khong dung de thay mot role duy nhat neu SOP/WI dang ap cho pham vi hep va da xac dinh duoc actor cu the.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>POU_LEADS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Point-of-Use Leads</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Nhom dau moi tai diem dung</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>WKM, SL, QCL, SCM</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Dung khi can goi lop actor kiem tai lieu, dung cu, vat tu va quy tac tai diem dung.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Khong dung de thay owner cua toan bo du lieu nghiep vu hoac owner phong ban.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>QUALITY_CORE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Quality Core</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Nhom nong cot chat luong</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>QA, QE, QCL, QC, QMS, MCS</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Dung khi tai lieu can gom nhom role cot loi cho inspection, release, NCR/CAPA va measurement confidence.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Khong dung de thay QA khi tai lieu dang noi toi final authority cua bo phan chat luong.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SUPPORT_ENABLEMENT</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Support Enablement Functions</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Nhom chuc nang ho tro nen</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>mixed bundle</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>SCM, D-FIN, D-HR, D-EHS, D-IT, D-ERP</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Dung khi can gom nhom chuc nang ho tro vat tu, tai chinh, nhan su, an toan, CNTT va ERP de mo ta lop enablement chung.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Khong dung de thay the D-code hoac role cu the khi tai lieu da biet ro bo phan nao dang nhan viec.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SYSTEM_OWNERS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>System Owners</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Nhom so huu he thong</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ITA, ESA</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Dung khi tai lieu dang noi toi lop actor so huu nen tang he thong, quyen truy cap, tich hop va cau hinh ky thuat.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Khong dung de che mo owner du lieu nghiep vu hoac thay the named admin da duoc chi ro.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TOP_MGMT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Top Management</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ban lanh dao</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>role bundle</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>CEO, PD, QA[QMR], ENGM, SCM, FIN</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Dung cho lop lanh dao cap cao trong xem xet cua lanh dao, ra quyet dinh chien luoc va escalations cap cao.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Khong dung thay role phe duyet cu the khi ANNEX-120 da chi ro ai giu authority.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/04-RACI-Authority/role-and-department-bundles.html</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7899,7 +8861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8240,17 +9202,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>D-PPC</t>
+          <t>D-MNT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Production Planning and Control Function</t>
+          <t>Maintenance Function</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Dieu do va kiem soat san xuat</t>
+          <t>Bo phan Bao tri</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -8270,7 +9232,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>PPL, PD, WKM</t>
+          <t>MNT, WKM, PD</t>
         </is>
       </c>
     </row>
@@ -8280,24 +9242,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>D-PPC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Production Planning and Control Function</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Dieu do va kiem soat san xuat</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>D-PROD</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Production Department</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Phong San xuat</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>department</t>
-        </is>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-production-handbook.html</t>
@@ -8305,7 +9272,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>PD, WKM, SL</t>
+          <t>PPL, PD, WKM</t>
         </is>
       </c>
     </row>
@@ -8315,37 +9282,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>D-PUR</t>
+          <t>D-PROD</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Purchasing Function</t>
+          <t>Production Department</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bo phan Mua hang</t>
+          <t>Phong San xuat</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>subfunction</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>D-SCM</t>
+          <t>department</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-production-handbook.html</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>BUY, SCM</t>
+          <t>PD, WKM, SL</t>
         </is>
       </c>
     </row>
@@ -8355,32 +9317,37 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>D-QUAL</t>
+          <t>D-PUR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Quality Department</t>
+          <t>Purchasing Function</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Phong Chat luong</t>
+          <t>Bo phan Mua hang</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>department</t>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-quality-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>QA, QMS, QE, QCL, MCS</t>
+          <t>BUY, SCM</t>
         </is>
       </c>
     </row>
@@ -8390,17 +9357,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>D-SCM</t>
+          <t>D-QUAL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Supply Chain Department</t>
+          <t>Quality Department</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Phong Chuoi cung ung</t>
+          <t>Phong Chat luong</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -8410,12 +9377,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-quality-handbook.html</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SCM, BUY, WAR, TOOL, LOG</t>
+          <t>QA, QMS, QE, QCL, MCS</t>
         </is>
       </c>
     </row>
@@ -8425,17 +9392,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>D-SCS</t>
+          <t>D-SCM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sales and Customer Service Department</t>
+          <t>Supply Chain Department</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Phong Kinh doanh va Dich vu khach hang</t>
+          <t>Phong Chuoi cung ung</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -8445,12 +9412,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-sales-and-customer-service-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CS, EST</t>
+          <t>SCM, BUY, WAR, TOOL, LOG</t>
         </is>
       </c>
     </row>
@@ -8460,37 +9427,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>D-TCR</t>
+          <t>D-SCS</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tool Crib Function</t>
+          <t>Sales and Customer Service Department</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bo phan Kho dao cu</t>
+          <t>Phong Kinh doanh va Dich vu khach hang</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>subfunction</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>D-SCM</t>
+          <t>department</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-sales-and-customer-service-handbook.html</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TOOL, SCM</t>
+          <t>CS, EST</t>
         </is>
       </c>
     </row>
@@ -8500,35 +9462,75 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>D-TCR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Tool Crib Function</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Bo phan Kho dao cu</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>subfunction</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>D-SCM</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>TOOL, SCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>D-WHS</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Warehouse Function</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Bo phan Kho</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>subfunction</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>D-SCM</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>02-Tai-Lieu-He-Thong/03-Organization/02-Department-Handbooks/dept-supply-chain-handbook.html</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>WAR, SCM</t>
         </is>

</xml_diff>